<commit_message>
Pending changes exported from your codespace
</commit_message>
<xml_diff>
--- a/fuction_ensemble_3/media_ponderada/comparacao_mse_50_ensembles.xlsx
+++ b/fuction_ensemble_3/media_ponderada/comparacao_mse_50_ensembles.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E51"/>
+  <dimension ref="A1:F51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -451,7 +451,12 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>num_redes_restantes</t>
+          <t>num_redes_filtradas</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>nome_redes_filtradas</t>
         </is>
       </c>
     </row>
@@ -471,6 +476,11 @@
       <c r="E2" t="n">
         <v>2</v>
       </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>['1000_model_28_9_21.xlsx', '1000_model_31_9_8.xlsx']</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -487,6 +497,11 @@
       </c>
       <c r="E3" t="n">
         <v>2</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>['1000_model_28_9_21.xlsx', '1000_model_31_9_8.xlsx']</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -505,6 +520,11 @@
       <c r="E4" t="n">
         <v>2</v>
       </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>['1000_model_28_9_21.xlsx', '1000_model_31_9_8.xlsx']</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -522,6 +542,11 @@
       <c r="E5" t="n">
         <v>2</v>
       </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>['1000_model_28_9_21.xlsx', '1000_model_31_9_8.xlsx']</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -539,6 +564,11 @@
       <c r="E6" t="n">
         <v>2</v>
       </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>['1000_model_28_9_21.xlsx', '1000_model_31_9_8.xlsx']</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -556,6 +586,11 @@
       <c r="E7" t="n">
         <v>2</v>
       </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>['1000_model_28_9_21.xlsx', '1000_model_31_9_8.xlsx']</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -573,6 +608,11 @@
       <c r="E8" t="n">
         <v>2</v>
       </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>['1000_model_28_9_21.xlsx', '1000_model_31_9_8.xlsx']</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -590,6 +630,11 @@
       <c r="E9" t="n">
         <v>2</v>
       </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>['1000_model_28_9_21.xlsx', '1000_model_31_9_8.xlsx']</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -607,6 +652,11 @@
       <c r="E10" t="n">
         <v>2</v>
       </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>['1000_model_28_9_21.xlsx', '1000_model_31_9_8.xlsx']</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -623,6 +673,11 @@
       </c>
       <c r="E11" t="n">
         <v>2</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>['1000_model_28_9_21.xlsx', '1000_model_31_9_8.xlsx']</t>
+        </is>
       </c>
     </row>
     <row r="12">
@@ -641,6 +696,11 @@
       <c r="E12" t="n">
         <v>2</v>
       </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>['1000_model_28_9_21.xlsx', '1000_model_31_9_8.xlsx']</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -658,6 +718,11 @@
       <c r="E13" t="n">
         <v>2</v>
       </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>['1000_model_28_9_21.xlsx', '1000_model_31_9_8.xlsx']</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -675,6 +740,11 @@
       <c r="E14" t="n">
         <v>2</v>
       </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>['1000_model_31_9_8.xlsx', '1000_model_8_4_3.xlsx']</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -692,6 +762,11 @@
       <c r="E15" t="n">
         <v>2</v>
       </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>['1000_model_31_9_8.xlsx', '1000_model_8_4_3.xlsx']</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -709,6 +784,11 @@
       <c r="E16" t="n">
         <v>2</v>
       </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>['1000_model_28_9_21.xlsx', '1000_model_31_9_8.xlsx']</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -726,6 +806,11 @@
       <c r="E17" t="n">
         <v>2</v>
       </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>['1000_model_28_9_21.xlsx', '1000_model_31_9_8.xlsx']</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -743,6 +828,11 @@
       <c r="E18" t="n">
         <v>2</v>
       </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>['1000_model_28_9_21.xlsx', '1000_model_31_9_8.xlsx']</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -760,6 +850,11 @@
       <c r="E19" t="n">
         <v>2</v>
       </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>['1000_model_28_9_21.xlsx', '1000_model_31_9_8.xlsx']</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -777,6 +872,11 @@
       <c r="E20" t="n">
         <v>2</v>
       </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>['1000_model_28_9_21.xlsx', '1000_model_31_9_8.xlsx']</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -794,6 +894,11 @@
       <c r="E21" t="n">
         <v>2</v>
       </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>['1000_model_28_9_21.xlsx', '1000_model_31_9_8.xlsx']</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -811,6 +916,11 @@
       <c r="E22" t="n">
         <v>2</v>
       </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>['1000_model_28_9_21.xlsx', '1000_model_31_9_8.xlsx']</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -828,6 +938,11 @@
       <c r="E23" t="n">
         <v>2</v>
       </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>['1000_model_28_9_21.xlsx', '1000_model_31_9_8.xlsx']</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -845,6 +960,11 @@
       <c r="E24" t="n">
         <v>2</v>
       </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>['1000_model_28_9_21.xlsx', '1000_model_31_9_8.xlsx']</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -862,6 +982,11 @@
       <c r="E25" t="n">
         <v>3</v>
       </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>['1000_model_26_8_14.xlsx', '1000_model_31_9_8.xlsx', '1000_model_36_5_0.xlsx']</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -879,6 +1004,11 @@
       <c r="E26" t="n">
         <v>2</v>
       </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>['1000_model_31_9_8.xlsx', '1000_model_8_4_3.xlsx']</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -896,6 +1026,11 @@
       <c r="E27" t="n">
         <v>2</v>
       </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>['1000_model_31_9_8.xlsx', '1000_model_8_4_3.xlsx']</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -913,6 +1048,11 @@
       <c r="E28" t="n">
         <v>2</v>
       </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>['1000_model_31_9_8.xlsx', '1000_model_8_4_3.xlsx']</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -930,6 +1070,11 @@
       <c r="E29" t="n">
         <v>2</v>
       </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>['1000_model_31_9_8.xlsx', '1000_model_8_4_3.xlsx']</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -947,6 +1092,11 @@
       <c r="E30" t="n">
         <v>2</v>
       </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>['1000_model_31_9_8.xlsx', '1000_model_8_4_3.xlsx']</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -964,6 +1114,11 @@
       <c r="E31" t="n">
         <v>2</v>
       </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>['1000_model_31_9_8.xlsx', '1000_model_8_4_3.xlsx']</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -981,6 +1136,11 @@
       <c r="E32" t="n">
         <v>2</v>
       </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>['1000_model_31_9_8.xlsx', '1000_model_8_4_3.xlsx']</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -998,6 +1158,11 @@
       <c r="E33" t="n">
         <v>2</v>
       </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>['1000_model_31_9_8.xlsx', '1000_model_8_4_3.xlsx']</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -1015,6 +1180,11 @@
       <c r="E34" t="n">
         <v>2</v>
       </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>['1000_model_31_9_8.xlsx', '1000_model_8_4_3.xlsx']</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -1032,6 +1202,11 @@
       <c r="E35" t="n">
         <v>2</v>
       </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>['1000_model_31_9_8.xlsx', '1000_model_8_4_3.xlsx']</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -1049,6 +1224,11 @@
       <c r="E36" t="n">
         <v>2</v>
       </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>['1000_model_31_9_8.xlsx', '1000_model_8_4_3.xlsx']</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -1066,6 +1246,11 @@
       <c r="E37" t="n">
         <v>2</v>
       </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>['1000_model_31_9_8.xlsx', '1000_model_8_4_3.xlsx']</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -1083,6 +1268,11 @@
       <c r="E38" t="n">
         <v>2</v>
       </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>['1000_model_31_9_8.xlsx', '1000_model_8_4_3.xlsx']</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -1100,6 +1290,11 @@
       <c r="E39" t="n">
         <v>2</v>
       </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>['1000_model_31_9_8.xlsx', '1000_model_8_4_3.xlsx']</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -1117,6 +1312,11 @@
       <c r="E40" t="n">
         <v>2</v>
       </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>['1000_model_31_9_8.xlsx', '1000_model_8_4_3.xlsx']</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -1134,6 +1334,11 @@
       <c r="E41" t="n">
         <v>2</v>
       </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>['1000_model_31_9_8.xlsx', '1000_model_8_4_3.xlsx']</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -1151,6 +1356,11 @@
       <c r="E42" t="n">
         <v>2</v>
       </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>['1000_model_31_9_8.xlsx', '1000_model_8_4_3.xlsx']</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -1168,6 +1378,11 @@
       <c r="E43" t="n">
         <v>2</v>
       </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>['1000_model_31_9_8.xlsx', '1000_model_8_4_3.xlsx']</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -1185,6 +1400,11 @@
       <c r="E44" t="n">
         <v>2</v>
       </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>['1000_model_31_9_8.xlsx', '1000_model_8_4_3.xlsx']</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -1202,6 +1422,11 @@
       <c r="E45" t="n">
         <v>2</v>
       </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>['1000_model_31_9_8.xlsx', '1000_model_8_4_3.xlsx']</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -1219,6 +1444,11 @@
       <c r="E46" t="n">
         <v>2</v>
       </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>['1000_model_31_9_8.xlsx', '1000_model_8_4_3.xlsx']</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -1236,6 +1466,11 @@
       <c r="E47" t="n">
         <v>2</v>
       </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>['1000_model_31_9_8.xlsx', '1000_model_8_4_3.xlsx']</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -1253,6 +1488,11 @@
       <c r="E48" t="n">
         <v>2</v>
       </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>['1000_model_31_9_8.xlsx', '1000_model_8_4_3.xlsx']</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -1270,6 +1510,11 @@
       <c r="E49" t="n">
         <v>2</v>
       </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>['1000_model_31_9_8.xlsx', '1000_model_8_4_3.xlsx']</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -1287,6 +1532,11 @@
       <c r="E50" t="n">
         <v>2</v>
       </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>['1000_model_28_9_21.xlsx', '1000_model_31_9_8.xlsx']</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -1303,6 +1553,11 @@
       </c>
       <c r="E51" t="n">
         <v>2</v>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>['1000_model_31_9_8.xlsx', '1000_model_8_4_3.xlsx']</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>